<commit_message>
update code and data
</commit_message>
<xml_diff>
--- a/thermal.xlsx
+++ b/thermal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joaobiosmac/Desktop/Artigo BEPE/Data and code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joaobiosmac/Desktop/Projeto 1 BEPE/BEPE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A83F4162-0F8C-ED42-B51D-EFB91AF0E2AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7FD507A-B6BC-1947-B2F2-039E3CD3FE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1980" yWindow="600" windowWidth="26020" windowHeight="14300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>Species</t>
   </si>
@@ -73,63 +73,12 @@
     <t>Synbranchus marmoratus</t>
   </si>
   <si>
-    <t>ARR</t>
-  </si>
-  <si>
-    <t>1.09</t>
-  </si>
-  <si>
-    <t>3.88</t>
-  </si>
-  <si>
-    <t>0.61</t>
-  </si>
-  <si>
-    <t>0.78</t>
-  </si>
-  <si>
-    <t>0.82</t>
-  </si>
-  <si>
-    <t>0.79</t>
-  </si>
-  <si>
     <t>Geophagus iporangensis</t>
   </si>
   <si>
     <t>Atlantirivulus peruibensis</t>
   </si>
   <si>
-    <t>1.88</t>
-  </si>
-  <si>
-    <t>0.39</t>
-  </si>
-  <si>
-    <t>1.52</t>
-  </si>
-  <si>
-    <t>2.17</t>
-  </si>
-  <si>
-    <t>0.75</t>
-  </si>
-  <si>
-    <t>0.91</t>
-  </si>
-  <si>
-    <t>2.46</t>
-  </si>
-  <si>
-    <t>2.48</t>
-  </si>
-  <si>
-    <t>0.86</t>
-  </si>
-  <si>
-    <t>2.77</t>
-  </si>
-  <si>
     <t>CTMax</t>
   </si>
   <si>
@@ -212,9 +161,6 @@
   </si>
   <si>
     <t>7.45</t>
-  </si>
-  <si>
-    <t>0.31</t>
   </si>
   <si>
     <t>37.48</t>
@@ -331,7 +277,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -344,12 +290,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -659,280 +599,222 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.6640625" customWidth="1"/>
     <col min="2" max="2" width="23.33203125" customWidth="1"/>
     <col min="3" max="3" width="24.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20" style="6" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B2" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B7" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B9" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B10" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="C13" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B15" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B16" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B18" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>21</v>
+      <c r="B19" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>